<commit_message>
chg: Added Bardufoss frequencies to master comm spreadsheet
</commit_message>
<xml_diff>
--- a/COMMUNICATIONS/TRMA Frequency and callsign master list.xlsx
+++ b/COMMUNICATIONS/TRMA Frequency and callsign master list.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2275" uniqueCount="1361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2289" uniqueCount="1369">
   <si>
     <t>AWACS</t>
   </si>
@@ -4107,6 +4107,30 @@
   </si>
   <si>
     <t>Saber</t>
+  </si>
+  <si>
+    <t>ma</t>
+  </si>
+  <si>
+    <t>Bardufoss</t>
+  </si>
+  <si>
+    <t>250.65</t>
+  </si>
+  <si>
+    <t>118.100</t>
+  </si>
+  <si>
+    <t>251.65</t>
+  </si>
+  <si>
+    <t>252.75</t>
+  </si>
+  <si>
+    <t>250.8</t>
+  </si>
+  <si>
+    <t>118.0</t>
   </si>
 </sst>
 </file>
@@ -6039,7 +6063,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="428">
+  <cellXfs count="430">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -6761,6 +6785,8 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="89" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -7470,7 +7496,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr codeName="Ark1"/>
-  <dimension ref="A1:AP83"/>
+  <dimension ref="A1:AP86"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="16" max="16" width="13.5703125" customWidth="1"/>
@@ -7575,13 +7601,13 @@
       <c r="N2" s="107" t="s">
         <v>330</v>
       </c>
-      <c r="V2" s="296" t="s">
+      <c r="V2" s="298" t="s">
         <v>0</v>
       </c>
-      <c r="W2" s="296"/>
-      <c r="X2" s="296"/>
-      <c r="Y2" s="296"/>
-      <c r="Z2" s="296"/>
+      <c r="W2" s="298"/>
+      <c r="X2" s="298"/>
+      <c r="Y2" s="298"/>
+      <c r="Z2" s="298"/>
     </row>
     <row r="3" spans="1:42">
       <c r="A3" s="107" t="s">
@@ -7630,9 +7656,9 @@
       <c r="P3" t="s">
         <v>426</v>
       </c>
-      <c r="R3" s="295"/>
-      <c r="S3" s="295"/>
-      <c r="T3" s="295"/>
+      <c r="R3" s="297"/>
+      <c r="S3" s="297"/>
+      <c r="T3" s="297"/>
       <c r="V3" s="101" t="s">
         <v>328</v>
       </c>
@@ -7714,22 +7740,22 @@
       <c r="AA4" s="23"/>
       <c r="AB4" s="23"/>
       <c r="AC4" s="23"/>
-      <c r="AD4" s="296" t="s">
+      <c r="AD4" s="298" t="s">
         <v>429</v>
       </c>
-      <c r="AE4" s="296"/>
-      <c r="AF4" s="296"/>
-      <c r="AG4" s="296"/>
-      <c r="AH4" s="296"/>
-      <c r="AJ4" s="296" t="s">
+      <c r="AE4" s="298"/>
+      <c r="AF4" s="298"/>
+      <c r="AG4" s="298"/>
+      <c r="AH4" s="298"/>
+      <c r="AJ4" s="298" t="s">
         <v>1</v>
       </c>
-      <c r="AK4" s="296"/>
-      <c r="AL4" s="296"/>
-      <c r="AM4" s="296"/>
-      <c r="AN4" s="296"/>
-      <c r="AO4" s="296"/>
-      <c r="AP4" s="296"/>
+      <c r="AK4" s="298"/>
+      <c r="AL4" s="298"/>
+      <c r="AM4" s="298"/>
+      <c r="AN4" s="298"/>
+      <c r="AO4" s="298"/>
+      <c r="AP4" s="298"/>
     </row>
     <row r="5" spans="1:42" ht="15.75">
       <c r="A5" s="107" t="s">
@@ -8966,15 +8992,15 @@
       <c r="AH18" s="3" t="s">
         <v>472</v>
       </c>
-      <c r="AJ18" s="296" t="s">
+      <c r="AJ18" s="298" t="s">
         <v>274</v>
       </c>
-      <c r="AK18" s="296"/>
-      <c r="AL18" s="296"/>
-      <c r="AM18" s="296"/>
-      <c r="AN18" s="296"/>
-      <c r="AO18" s="296"/>
-      <c r="AP18" s="296"/>
+      <c r="AK18" s="298"/>
+      <c r="AL18" s="298"/>
+      <c r="AM18" s="298"/>
+      <c r="AN18" s="298"/>
+      <c r="AO18" s="298"/>
+      <c r="AP18" s="298"/>
     </row>
     <row r="19" spans="1:42" ht="15.75">
       <c r="A19" s="107" t="s">
@@ -9107,9 +9133,9 @@
       </c>
       <c r="P20" s="2"/>
       <c r="Q20" s="2"/>
-      <c r="R20" s="295"/>
-      <c r="S20" s="295"/>
-      <c r="T20" s="295"/>
+      <c r="R20" s="297"/>
+      <c r="S20" s="297"/>
+      <c r="T20" s="297"/>
       <c r="U20" s="2"/>
       <c r="V20" s="271" t="s">
         <v>1252</v>
@@ -9464,6 +9490,9 @@
       </c>
       <c r="O24" s="2"/>
       <c r="P24" s="2"/>
+      <c r="Y24" t="s">
+        <v>1361</v>
+      </c>
       <c r="AJ24" s="116" t="s">
         <v>552</v>
       </c>
@@ -9532,13 +9561,13 @@
       <c r="R25" s="24"/>
       <c r="S25" s="24"/>
       <c r="T25" s="24"/>
-      <c r="AD25" s="296" t="s">
+      <c r="AD25" s="298" t="s">
         <v>486</v>
       </c>
-      <c r="AE25" s="296"/>
-      <c r="AF25" s="296"/>
-      <c r="AG25" s="296"/>
-      <c r="AH25" s="296"/>
+      <c r="AE25" s="298"/>
+      <c r="AF25" s="298"/>
+      <c r="AG25" s="298"/>
+      <c r="AH25" s="298"/>
       <c r="AJ25" s="116" t="s">
         <v>555</v>
       </c>
@@ -9808,15 +9837,15 @@
       <c r="N29" s="107" t="s">
         <v>355</v>
       </c>
-      <c r="V29" s="296" t="s">
+      <c r="V29" s="298" t="s">
         <v>212</v>
       </c>
-      <c r="W29" s="296"/>
-      <c r="X29" s="296"/>
-      <c r="Y29" s="296"/>
-      <c r="Z29" s="296"/>
-      <c r="AA29" s="296"/>
-      <c r="AB29" s="296"/>
+      <c r="W29" s="298"/>
+      <c r="X29" s="298"/>
+      <c r="Y29" s="298"/>
+      <c r="Z29" s="298"/>
+      <c r="AA29" s="298"/>
+      <c r="AB29" s="298"/>
     </row>
     <row r="30" spans="1:42">
       <c r="A30" s="107"/>
@@ -9872,15 +9901,15 @@
       </c>
       <c r="AA30" s="29"/>
       <c r="AB30" s="29"/>
-      <c r="AJ30" s="296" t="s">
+      <c r="AJ30" s="298" t="s">
         <v>831</v>
       </c>
-      <c r="AK30" s="296"/>
-      <c r="AL30" s="296"/>
-      <c r="AM30" s="296"/>
-      <c r="AN30" s="296"/>
-      <c r="AO30" s="296"/>
-      <c r="AP30" s="296"/>
+      <c r="AK30" s="298"/>
+      <c r="AL30" s="298"/>
+      <c r="AM30" s="298"/>
+      <c r="AN30" s="298"/>
+      <c r="AO30" s="298"/>
+      <c r="AP30" s="298"/>
     </row>
     <row r="31" spans="1:42">
       <c r="B31" s="24"/>
@@ -9967,15 +9996,15 @@
       <c r="AJ34" s="23"/>
     </row>
     <row r="37" spans="22:36">
-      <c r="V37" s="296" t="s">
+      <c r="V37" s="298" t="s">
         <v>9</v>
       </c>
-      <c r="W37" s="296"/>
-      <c r="X37" s="296"/>
-      <c r="Y37" s="296"/>
-      <c r="Z37" s="296"/>
-      <c r="AA37" s="296"/>
-      <c r="AB37" s="296"/>
+      <c r="W37" s="298"/>
+      <c r="X37" s="298"/>
+      <c r="Y37" s="298"/>
+      <c r="Z37" s="298"/>
+      <c r="AA37" s="298"/>
+      <c r="AB37" s="298"/>
     </row>
     <row r="38" spans="22:36">
       <c r="V38" s="29" t="s">
@@ -9995,11 +10024,11 @@
       </c>
       <c r="AA38" s="29"/>
       <c r="AB38" s="29"/>
-      <c r="AD38" s="297" t="s">
+      <c r="AD38" s="299" t="s">
         <v>260</v>
       </c>
-      <c r="AE38" s="298"/>
-      <c r="AF38" s="299"/>
+      <c r="AE38" s="300"/>
+      <c r="AF38" s="301"/>
     </row>
     <row r="39" spans="22:36">
       <c r="V39" s="3" t="s">
@@ -10036,15 +10065,15 @@
       <c r="AF41" s="3"/>
     </row>
     <row r="42" spans="22:36">
-      <c r="V42" s="296" t="s">
+      <c r="V42" s="298" t="s">
         <v>244</v>
       </c>
-      <c r="W42" s="296"/>
-      <c r="X42" s="296"/>
-      <c r="Y42" s="296"/>
-      <c r="Z42" s="296"/>
-      <c r="AA42" s="296"/>
-      <c r="AB42" s="296"/>
+      <c r="W42" s="298"/>
+      <c r="X42" s="298"/>
+      <c r="Y42" s="298"/>
+      <c r="Z42" s="298"/>
+      <c r="AA42" s="298"/>
+      <c r="AB42" s="298"/>
       <c r="AD42" s="3" t="s">
         <v>254</v>
       </c>
@@ -10114,15 +10143,15 @@
       <c r="AF47" s="3"/>
     </row>
     <row r="48" spans="22:36">
-      <c r="V48" s="300" t="s">
+      <c r="V48" s="302" t="s">
         <v>473</v>
       </c>
-      <c r="W48" s="301"/>
-      <c r="X48" s="301"/>
-      <c r="Y48" s="301"/>
-      <c r="Z48" s="301"/>
-      <c r="AA48" s="301"/>
-      <c r="AB48" s="302"/>
+      <c r="W48" s="303"/>
+      <c r="X48" s="303"/>
+      <c r="Y48" s="303"/>
+      <c r="Z48" s="303"/>
+      <c r="AA48" s="303"/>
+      <c r="AB48" s="304"/>
       <c r="AD48" s="3" t="s">
         <v>261</v>
       </c>
@@ -10336,8 +10365,12 @@
       <c r="W59" s="231" t="s">
         <v>908</v>
       </c>
-      <c r="X59" s="231"/>
-      <c r="Y59" s="231"/>
+      <c r="X59" s="231" t="s">
+        <v>1367</v>
+      </c>
+      <c r="Y59" s="231" t="s">
+        <v>1368</v>
+      </c>
       <c r="Z59" s="231"/>
       <c r="AA59" s="231"/>
       <c r="AB59" s="232"/>
@@ -10729,6 +10762,45 @@
       <c r="Z83" s="231"/>
       <c r="AA83" s="231"/>
       <c r="AB83" s="232"/>
+    </row>
+    <row r="84" spans="22:28">
+      <c r="V84" s="295" t="s">
+        <v>1362</v>
+      </c>
+      <c r="W84" s="226" t="s">
+        <v>906</v>
+      </c>
+      <c r="X84" s="296" t="s">
+        <v>1365</v>
+      </c>
+      <c r="AB84" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="85" spans="22:28">
+      <c r="V85" s="295" t="s">
+        <v>1362</v>
+      </c>
+      <c r="W85" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="X85" s="296" t="s">
+        <v>1366</v>
+      </c>
+    </row>
+    <row r="86" spans="22:28" ht="15.75" thickBot="1">
+      <c r="V86" s="295" t="s">
+        <v>1362</v>
+      </c>
+      <c r="W86" s="231" t="s">
+        <v>908</v>
+      </c>
+      <c r="X86" t="s">
+        <v>1363</v>
+      </c>
+      <c r="Y86" t="s">
+        <v>1364</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -10767,40 +10839,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="393" t="s">
+      <c r="A1" s="395" t="s">
         <v>487</v>
       </c>
-      <c r="B1" s="394"/>
-      <c r="C1" s="394"/>
-      <c r="D1" s="394"/>
-      <c r="E1" s="394"/>
-      <c r="F1" s="394"/>
-      <c r="G1" s="394"/>
-      <c r="H1" s="395"/>
+      <c r="B1" s="396"/>
+      <c r="C1" s="396"/>
+      <c r="D1" s="396"/>
+      <c r="E1" s="396"/>
+      <c r="F1" s="396"/>
+      <c r="G1" s="396"/>
+      <c r="H1" s="397"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" thickBot="1">
-      <c r="A2" s="396"/>
-      <c r="B2" s="397"/>
-      <c r="C2" s="397"/>
-      <c r="D2" s="397"/>
-      <c r="E2" s="397"/>
-      <c r="F2" s="397"/>
-      <c r="G2" s="397"/>
-      <c r="H2" s="398"/>
+      <c r="A2" s="398"/>
+      <c r="B2" s="399"/>
+      <c r="C2" s="399"/>
+      <c r="D2" s="399"/>
+      <c r="E2" s="399"/>
+      <c r="F2" s="399"/>
+      <c r="G2" s="399"/>
+      <c r="H2" s="400"/>
     </row>
     <row r="3" spans="1:8" ht="21" thickBot="1">
-      <c r="A3" s="399" t="s">
+      <c r="A3" s="401" t="s">
         <v>751</v>
       </c>
-      <c r="B3" s="400"/>
-      <c r="C3" s="400"/>
-      <c r="D3" s="401"/>
-      <c r="E3" s="399" t="s">
+      <c r="B3" s="402"/>
+      <c r="C3" s="402"/>
+      <c r="D3" s="403"/>
+      <c r="E3" s="401" t="s">
         <v>221</v>
       </c>
-      <c r="F3" s="400"/>
-      <c r="G3" s="400"/>
-      <c r="H3" s="401"/>
+      <c r="F3" s="402"/>
+      <c r="G3" s="402"/>
+      <c r="H3" s="403"/>
     </row>
     <row r="4" spans="1:8" ht="16.5">
       <c r="A4" s="166">
@@ -11273,18 +11345,18 @@
       <c r="H24" s="146"/>
     </row>
     <row r="25" spans="1:8" ht="20.25" thickBot="1">
-      <c r="A25" s="402" t="s">
+      <c r="A25" s="404" t="s">
         <v>314</v>
       </c>
-      <c r="B25" s="403"/>
-      <c r="C25" s="403"/>
-      <c r="D25" s="404"/>
-      <c r="E25" s="402" t="s">
+      <c r="B25" s="405"/>
+      <c r="C25" s="405"/>
+      <c r="D25" s="406"/>
+      <c r="E25" s="404" t="s">
         <v>801</v>
       </c>
-      <c r="F25" s="403"/>
-      <c r="G25" s="403"/>
-      <c r="H25" s="404"/>
+      <c r="F25" s="405"/>
+      <c r="G25" s="405"/>
+      <c r="H25" s="406"/>
     </row>
     <row r="26" spans="1:8" ht="16.5">
       <c r="A26" s="155">
@@ -11694,40 +11766,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1">
-      <c r="A1" s="422" t="s">
+      <c r="A1" s="424" t="s">
         <v>326</v>
       </c>
-      <c r="B1" s="422"/>
-      <c r="C1" s="422"/>
-      <c r="D1" s="422"/>
-      <c r="E1" s="422"/>
-      <c r="F1" s="422"/>
-      <c r="G1" s="422"/>
-      <c r="H1" s="422"/>
+      <c r="B1" s="424"/>
+      <c r="C1" s="424"/>
+      <c r="D1" s="424"/>
+      <c r="E1" s="424"/>
+      <c r="F1" s="424"/>
+      <c r="G1" s="424"/>
+      <c r="H1" s="424"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A2" s="423"/>
-      <c r="B2" s="423"/>
-      <c r="C2" s="423"/>
-      <c r="D2" s="423"/>
-      <c r="E2" s="423"/>
-      <c r="F2" s="423"/>
-      <c r="G2" s="423"/>
-      <c r="H2" s="423"/>
+      <c r="A2" s="425"/>
+      <c r="B2" s="425"/>
+      <c r="C2" s="425"/>
+      <c r="D2" s="425"/>
+      <c r="E2" s="425"/>
+      <c r="F2" s="425"/>
+      <c r="G2" s="425"/>
+      <c r="H2" s="425"/>
     </row>
     <row r="3" spans="1:8" ht="24" thickBot="1">
-      <c r="A3" s="424" t="s">
+      <c r="A3" s="426" t="s">
         <v>227</v>
       </c>
-      <c r="B3" s="425"/>
-      <c r="C3" s="426"/>
-      <c r="D3" s="427"/>
-      <c r="E3" s="424" t="s">
+      <c r="B3" s="427"/>
+      <c r="C3" s="428"/>
+      <c r="D3" s="429"/>
+      <c r="E3" s="426" t="s">
         <v>228</v>
       </c>
-      <c r="F3" s="425"/>
-      <c r="G3" s="426"/>
-      <c r="H3" s="427"/>
+      <c r="F3" s="427"/>
+      <c r="G3" s="428"/>
+      <c r="H3" s="429"/>
     </row>
     <row r="4" spans="1:8" ht="18">
       <c r="A4" s="31">
@@ -12020,114 +12092,114 @@
       <c r="H24" s="59"/>
     </row>
     <row r="25" spans="1:8" ht="24" thickBot="1">
-      <c r="A25" s="424" t="s">
+      <c r="A25" s="426" t="s">
         <v>289</v>
       </c>
-      <c r="B25" s="425"/>
-      <c r="C25" s="426"/>
-      <c r="D25" s="427"/>
-      <c r="E25" s="424" t="s">
+      <c r="B25" s="427"/>
+      <c r="C25" s="428"/>
+      <c r="D25" s="429"/>
+      <c r="E25" s="426" t="s">
         <v>290</v>
       </c>
-      <c r="F25" s="425"/>
-      <c r="G25" s="426"/>
-      <c r="H25" s="427"/>
+      <c r="F25" s="427"/>
+      <c r="G25" s="428"/>
+      <c r="H25" s="429"/>
     </row>
     <row r="26" spans="1:8" ht="18.75" thickBot="1">
       <c r="A26" s="35" t="s">
         <v>291</v>
       </c>
-      <c r="B26" s="411"/>
-      <c r="C26" s="412"/>
-      <c r="D26" s="413"/>
+      <c r="B26" s="413"/>
+      <c r="C26" s="414"/>
+      <c r="D26" s="415"/>
       <c r="E26" s="31" t="s">
         <v>292</v>
       </c>
-      <c r="F26" s="419"/>
-      <c r="G26" s="420"/>
-      <c r="H26" s="421"/>
+      <c r="F26" s="421"/>
+      <c r="G26" s="422"/>
+      <c r="H26" s="423"/>
     </row>
     <row r="27" spans="1:8" ht="18.75" thickBot="1">
       <c r="A27" s="43" t="s">
         <v>293</v>
       </c>
-      <c r="B27" s="414"/>
-      <c r="C27" s="415"/>
-      <c r="D27" s="417"/>
+      <c r="B27" s="416"/>
+      <c r="C27" s="417"/>
+      <c r="D27" s="419"/>
       <c r="E27" s="35" t="s">
         <v>294</v>
       </c>
-      <c r="F27" s="411"/>
-      <c r="G27" s="412"/>
-      <c r="H27" s="418"/>
+      <c r="F27" s="413"/>
+      <c r="G27" s="414"/>
+      <c r="H27" s="420"/>
     </row>
     <row r="28" spans="1:8" ht="18.75" thickBot="1">
       <c r="A28" s="35" t="s">
         <v>295</v>
       </c>
-      <c r="B28" s="411"/>
-      <c r="C28" s="412"/>
-      <c r="D28" s="413"/>
+      <c r="B28" s="413"/>
+      <c r="C28" s="414"/>
+      <c r="D28" s="415"/>
       <c r="E28" s="43" t="s">
         <v>296</v>
       </c>
-      <c r="F28" s="414"/>
-      <c r="G28" s="415"/>
-      <c r="H28" s="416"/>
+      <c r="F28" s="416"/>
+      <c r="G28" s="417"/>
+      <c r="H28" s="418"/>
     </row>
     <row r="29" spans="1:8" ht="18.75" thickBot="1">
       <c r="A29" s="43" t="s">
         <v>297</v>
       </c>
-      <c r="B29" s="414"/>
-      <c r="C29" s="415"/>
-      <c r="D29" s="417"/>
+      <c r="B29" s="416"/>
+      <c r="C29" s="417"/>
+      <c r="D29" s="419"/>
       <c r="E29" s="35" t="s">
         <v>298</v>
       </c>
-      <c r="F29" s="411"/>
-      <c r="G29" s="412"/>
-      <c r="H29" s="418"/>
+      <c r="F29" s="413"/>
+      <c r="G29" s="414"/>
+      <c r="H29" s="420"/>
     </row>
     <row r="30" spans="1:8" ht="18.75" thickBot="1">
       <c r="A30" s="35" t="s">
         <v>299</v>
       </c>
-      <c r="B30" s="411"/>
-      <c r="C30" s="412"/>
-      <c r="D30" s="413"/>
+      <c r="B30" s="413"/>
+      <c r="C30" s="414"/>
+      <c r="D30" s="415"/>
       <c r="E30" s="43" t="s">
         <v>300</v>
       </c>
-      <c r="F30" s="414"/>
-      <c r="G30" s="415"/>
-      <c r="H30" s="416"/>
+      <c r="F30" s="416"/>
+      <c r="G30" s="417"/>
+      <c r="H30" s="418"/>
     </row>
     <row r="31" spans="1:8" ht="18.75" thickBot="1">
       <c r="A31" s="43" t="s">
         <v>301</v>
       </c>
-      <c r="B31" s="414"/>
-      <c r="C31" s="415"/>
-      <c r="D31" s="417"/>
+      <c r="B31" s="416"/>
+      <c r="C31" s="417"/>
+      <c r="D31" s="419"/>
       <c r="E31" s="35" t="s">
         <v>302</v>
       </c>
-      <c r="F31" s="411"/>
-      <c r="G31" s="412"/>
-      <c r="H31" s="418"/>
+      <c r="F31" s="413"/>
+      <c r="G31" s="414"/>
+      <c r="H31" s="420"/>
     </row>
     <row r="32" spans="1:8" ht="18.75" thickBot="1">
       <c r="A32" s="35" t="s">
         <v>303</v>
       </c>
-      <c r="B32" s="411"/>
-      <c r="C32" s="412"/>
-      <c r="D32" s="413"/>
+      <c r="B32" s="413"/>
+      <c r="C32" s="414"/>
+      <c r="D32" s="415"/>
       <c r="E32" s="43"/>
-      <c r="F32" s="414"/>
-      <c r="G32" s="415"/>
-      <c r="H32" s="416" t="s">
+      <c r="F32" s="416"/>
+      <c r="G32" s="417"/>
+      <c r="H32" s="418" t="s">
         <v>242</v>
       </c>
     </row>
@@ -12135,13 +12207,13 @@
       <c r="A33" s="43" t="s">
         <v>304</v>
       </c>
-      <c r="B33" s="414"/>
-      <c r="C33" s="415"/>
-      <c r="D33" s="417"/>
+      <c r="B33" s="416"/>
+      <c r="C33" s="417"/>
+      <c r="D33" s="419"/>
       <c r="E33" s="35"/>
-      <c r="F33" s="411"/>
-      <c r="G33" s="412"/>
-      <c r="H33" s="418" t="s">
+      <c r="F33" s="413"/>
+      <c r="G33" s="414"/>
+      <c r="H33" s="420" t="s">
         <v>284</v>
       </c>
     </row>
@@ -12149,13 +12221,13 @@
       <c r="A34" s="35" t="s">
         <v>305</v>
       </c>
-      <c r="B34" s="411"/>
-      <c r="C34" s="412"/>
-      <c r="D34" s="413"/>
+      <c r="B34" s="413"/>
+      <c r="C34" s="414"/>
+      <c r="D34" s="415"/>
       <c r="E34" s="43"/>
-      <c r="F34" s="414"/>
-      <c r="G34" s="415"/>
-      <c r="H34" s="416" t="s">
+      <c r="F34" s="416"/>
+      <c r="G34" s="417"/>
+      <c r="H34" s="418" t="s">
         <v>285</v>
       </c>
     </row>
@@ -12163,13 +12235,13 @@
       <c r="A35" s="43" t="s">
         <v>306</v>
       </c>
-      <c r="B35" s="414"/>
-      <c r="C35" s="415"/>
-      <c r="D35" s="417"/>
+      <c r="B35" s="416"/>
+      <c r="C35" s="417"/>
+      <c r="D35" s="419"/>
       <c r="E35" s="35"/>
-      <c r="F35" s="411"/>
-      <c r="G35" s="412"/>
-      <c r="H35" s="418" t="s">
+      <c r="F35" s="413"/>
+      <c r="G35" s="414"/>
+      <c r="H35" s="420" t="s">
         <v>286</v>
       </c>
     </row>
@@ -12177,13 +12249,13 @@
       <c r="A36" s="35" t="s">
         <v>307</v>
       </c>
-      <c r="B36" s="411"/>
-      <c r="C36" s="412"/>
-      <c r="D36" s="413"/>
+      <c r="B36" s="413"/>
+      <c r="C36" s="414"/>
+      <c r="D36" s="415"/>
       <c r="E36" s="43"/>
-      <c r="F36" s="414"/>
-      <c r="G36" s="415"/>
-      <c r="H36" s="416" t="s">
+      <c r="F36" s="416"/>
+      <c r="G36" s="417"/>
+      <c r="H36" s="418" t="s">
         <v>287</v>
       </c>
     </row>
@@ -12191,13 +12263,13 @@
       <c r="A37" s="43" t="s">
         <v>308</v>
       </c>
-      <c r="B37" s="414"/>
-      <c r="C37" s="415"/>
-      <c r="D37" s="417"/>
+      <c r="B37" s="416"/>
+      <c r="C37" s="417"/>
+      <c r="D37" s="419"/>
       <c r="E37" s="35"/>
-      <c r="F37" s="411"/>
-      <c r="G37" s="412"/>
-      <c r="H37" s="418" t="s">
+      <c r="F37" s="413"/>
+      <c r="G37" s="414"/>
+      <c r="H37" s="420" t="s">
         <v>288</v>
       </c>
     </row>
@@ -12205,13 +12277,13 @@
       <c r="A38" s="35" t="s">
         <v>309</v>
       </c>
-      <c r="B38" s="411"/>
-      <c r="C38" s="412"/>
-      <c r="D38" s="413"/>
+      <c r="B38" s="413"/>
+      <c r="C38" s="414"/>
+      <c r="D38" s="415"/>
       <c r="E38" s="43"/>
-      <c r="F38" s="414"/>
-      <c r="G38" s="415"/>
-      <c r="H38" s="416" t="s">
+      <c r="F38" s="416"/>
+      <c r="G38" s="417"/>
+      <c r="H38" s="418" t="s">
         <v>241</v>
       </c>
     </row>
@@ -12219,13 +12291,13 @@
       <c r="A39" s="43" t="s">
         <v>310</v>
       </c>
-      <c r="B39" s="414"/>
-      <c r="C39" s="415"/>
-      <c r="D39" s="417"/>
+      <c r="B39" s="416"/>
+      <c r="C39" s="417"/>
+      <c r="D39" s="419"/>
       <c r="E39" s="35"/>
-      <c r="F39" s="411"/>
-      <c r="G39" s="412"/>
-      <c r="H39" s="418" t="s">
+      <c r="F39" s="413"/>
+      <c r="G39" s="414"/>
+      <c r="H39" s="420" t="s">
         <v>242</v>
       </c>
     </row>
@@ -12233,25 +12305,25 @@
       <c r="A40" s="35" t="s">
         <v>311</v>
       </c>
-      <c r="B40" s="411"/>
-      <c r="C40" s="412"/>
-      <c r="D40" s="413"/>
+      <c r="B40" s="413"/>
+      <c r="C40" s="414"/>
+      <c r="D40" s="415"/>
       <c r="E40" s="43"/>
-      <c r="F40" s="414"/>
-      <c r="G40" s="415"/>
-      <c r="H40" s="416"/>
+      <c r="F40" s="416"/>
+      <c r="G40" s="417"/>
+      <c r="H40" s="418"/>
     </row>
     <row r="41" spans="1:8" ht="18.75" thickBot="1">
       <c r="A41" s="55" t="s">
         <v>312</v>
       </c>
-      <c r="B41" s="405"/>
-      <c r="C41" s="406"/>
-      <c r="D41" s="407"/>
+      <c r="B41" s="407"/>
+      <c r="C41" s="408"/>
+      <c r="D41" s="409"/>
       <c r="E41" s="60"/>
-      <c r="F41" s="408"/>
-      <c r="G41" s="409"/>
-      <c r="H41" s="410"/>
+      <c r="F41" s="410"/>
+      <c r="G41" s="411"/>
+      <c r="H41" s="412"/>
     </row>
   </sheetData>
   <mergeCells count="37">
@@ -12342,55 +12414,55 @@
       </c>
     </row>
     <row r="2" spans="2:42">
-      <c r="B2" s="296" t="s">
+      <c r="B2" s="298" t="s">
         <v>276</v>
       </c>
-      <c r="C2" s="296"/>
-      <c r="D2" s="296"/>
-      <c r="E2" s="296"/>
-      <c r="F2" s="296"/>
-      <c r="H2" s="296" t="s">
+      <c r="C2" s="298"/>
+      <c r="D2" s="298"/>
+      <c r="E2" s="298"/>
+      <c r="F2" s="298"/>
+      <c r="H2" s="298" t="s">
         <v>1055</v>
       </c>
-      <c r="I2" s="296"/>
-      <c r="J2" s="296"/>
-      <c r="K2" s="296"/>
-      <c r="L2" s="296"/>
-      <c r="N2" s="296" t="s">
+      <c r="I2" s="298"/>
+      <c r="J2" s="298"/>
+      <c r="K2" s="298"/>
+      <c r="L2" s="298"/>
+      <c r="N2" s="298" t="s">
         <v>1054</v>
       </c>
-      <c r="O2" s="296"/>
-      <c r="P2" s="296"/>
-      <c r="Q2" s="296"/>
-      <c r="R2" s="296"/>
-      <c r="T2" s="296" t="s">
+      <c r="O2" s="298"/>
+      <c r="P2" s="298"/>
+      <c r="Q2" s="298"/>
+      <c r="R2" s="298"/>
+      <c r="T2" s="298" t="s">
         <v>236</v>
       </c>
-      <c r="U2" s="296"/>
-      <c r="V2" s="296"/>
-      <c r="W2" s="296"/>
-      <c r="X2" s="296"/>
-      <c r="Z2" s="296" t="s">
+      <c r="U2" s="298"/>
+      <c r="V2" s="298"/>
+      <c r="W2" s="298"/>
+      <c r="X2" s="298"/>
+      <c r="Z2" s="298" t="s">
         <v>246</v>
       </c>
-      <c r="AA2" s="296"/>
-      <c r="AB2" s="296"/>
-      <c r="AC2" s="296"/>
-      <c r="AD2" s="296"/>
-      <c r="AF2" s="296" t="s">
+      <c r="AA2" s="298"/>
+      <c r="AB2" s="298"/>
+      <c r="AC2" s="298"/>
+      <c r="AD2" s="298"/>
+      <c r="AF2" s="298" t="s">
         <v>317</v>
       </c>
-      <c r="AG2" s="296"/>
-      <c r="AH2" s="296"/>
-      <c r="AI2" s="296"/>
-      <c r="AJ2" s="296"/>
-      <c r="AL2" s="296" t="s">
+      <c r="AG2" s="298"/>
+      <c r="AH2" s="298"/>
+      <c r="AI2" s="298"/>
+      <c r="AJ2" s="298"/>
+      <c r="AL2" s="298" t="s">
         <v>491</v>
       </c>
-      <c r="AM2" s="296"/>
-      <c r="AN2" s="296"/>
-      <c r="AO2" s="296"/>
-      <c r="AP2" s="296"/>
+      <c r="AM2" s="298"/>
+      <c r="AN2" s="298"/>
+      <c r="AO2" s="298"/>
+      <c r="AP2" s="298"/>
     </row>
     <row r="3" spans="2:42">
       <c r="B3" s="101" t="s">
@@ -14105,20 +14177,20 @@
       <c r="X39" s="59"/>
     </row>
     <row r="41" spans="2:24">
-      <c r="B41" s="296" t="s">
+      <c r="B41" s="298" t="s">
         <v>697</v>
       </c>
-      <c r="C41" s="296"/>
-      <c r="D41" s="296"/>
-      <c r="E41" s="296"/>
-      <c r="F41" s="296"/>
-      <c r="H41" s="296" t="s">
+      <c r="C41" s="298"/>
+      <c r="D41" s="298"/>
+      <c r="E41" s="298"/>
+      <c r="F41" s="298"/>
+      <c r="H41" s="298" t="s">
         <v>750</v>
       </c>
-      <c r="I41" s="296"/>
-      <c r="J41" s="296"/>
-      <c r="K41" s="296"/>
-      <c r="L41" s="296"/>
+      <c r="I41" s="298"/>
+      <c r="J41" s="298"/>
+      <c r="K41" s="298"/>
+      <c r="L41" s="298"/>
     </row>
     <row r="42" spans="2:24">
       <c r="B42" s="101" t="s">
@@ -14700,39 +14772,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="27" customHeight="1" thickBot="1">
-      <c r="A1" s="315" t="s">
+      <c r="A1" s="317" t="s">
         <v>1351</v>
       </c>
-      <c r="B1" s="316"/>
-      <c r="C1" s="316"/>
-      <c r="D1" s="316"/>
-      <c r="E1" s="316"/>
-      <c r="F1" s="316"/>
-      <c r="G1" s="316"/>
-      <c r="H1" s="316"/>
-      <c r="I1" s="316"/>
-      <c r="J1" s="316"/>
-      <c r="K1" s="316"/>
-      <c r="L1" s="317"/>
+      <c r="B1" s="318"/>
+      <c r="C1" s="318"/>
+      <c r="D1" s="318"/>
+      <c r="E1" s="318"/>
+      <c r="F1" s="318"/>
+      <c r="G1" s="318"/>
+      <c r="H1" s="318"/>
+      <c r="I1" s="318"/>
+      <c r="J1" s="318"/>
+      <c r="K1" s="318"/>
+      <c r="L1" s="319"/>
     </row>
     <row r="2" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A2" s="312" t="s">
+      <c r="A2" s="314" t="s">
         <v>1146</v>
       </c>
-      <c r="B2" s="313"/>
-      <c r="C2" s="314"/>
+      <c r="B2" s="315"/>
+      <c r="C2" s="316"/>
       <c r="D2" s="258"/>
-      <c r="E2" s="312" t="s">
+      <c r="E2" s="314" t="s">
         <v>1055</v>
       </c>
-      <c r="F2" s="313"/>
-      <c r="G2" s="314"/>
+      <c r="F2" s="315"/>
+      <c r="G2" s="316"/>
       <c r="H2" s="258"/>
-      <c r="I2" s="312" t="s">
+      <c r="I2" s="314" t="s">
         <v>1054</v>
       </c>
-      <c r="J2" s="313"/>
-      <c r="K2" s="314"/>
+      <c r="J2" s="315"/>
+      <c r="K2" s="316"/>
       <c r="L2" s="122"/>
     </row>
     <row r="3" spans="1:12" ht="19.5" thickBot="1">
@@ -14768,7 +14840,7 @@
       <c r="L3" s="122"/>
     </row>
     <row r="4" spans="1:12" ht="18.75">
-      <c r="A4" s="306" t="s">
+      <c r="A4" s="308" t="s">
         <v>325</v>
       </c>
       <c r="B4" s="132" t="s">
@@ -14778,7 +14850,7 @@
         <v>705</v>
       </c>
       <c r="D4" s="253"/>
-      <c r="E4" s="309" t="s">
+      <c r="E4" s="311" t="s">
         <v>975</v>
       </c>
       <c r="F4" s="132" t="s">
@@ -14788,7 +14860,7 @@
         <v>1028</v>
       </c>
       <c r="H4" s="125"/>
-      <c r="I4" s="309" t="s">
+      <c r="I4" s="311" t="s">
         <v>1057</v>
       </c>
       <c r="J4" s="132" t="s">
@@ -14800,7 +14872,7 @@
       <c r="L4" s="122"/>
     </row>
     <row r="5" spans="1:12" ht="18.75">
-      <c r="A5" s="307"/>
+      <c r="A5" s="309"/>
       <c r="B5" s="131" t="s">
         <v>322</v>
       </c>
@@ -14808,7 +14880,7 @@
         <v>706</v>
       </c>
       <c r="D5" s="253"/>
-      <c r="E5" s="310"/>
+      <c r="E5" s="312"/>
       <c r="F5" s="131" t="s">
         <v>1002</v>
       </c>
@@ -14816,7 +14888,7 @@
         <v>1029</v>
       </c>
       <c r="H5" s="125"/>
-      <c r="I5" s="310"/>
+      <c r="I5" s="312"/>
       <c r="J5" s="131" t="s">
         <v>1092</v>
       </c>
@@ -14826,7 +14898,7 @@
       <c r="L5" s="122"/>
     </row>
     <row r="6" spans="1:12" ht="18.75">
-      <c r="A6" s="307"/>
+      <c r="A6" s="309"/>
       <c r="B6" s="131" t="s">
         <v>323</v>
       </c>
@@ -14834,7 +14906,7 @@
         <v>707</v>
       </c>
       <c r="D6" s="253"/>
-      <c r="E6" s="310"/>
+      <c r="E6" s="312"/>
       <c r="F6" s="131" t="s">
         <v>1003</v>
       </c>
@@ -14842,7 +14914,7 @@
         <v>1030</v>
       </c>
       <c r="H6" s="125"/>
-      <c r="I6" s="310"/>
+      <c r="I6" s="312"/>
       <c r="J6" s="131" t="s">
         <v>1093</v>
       </c>
@@ -14852,7 +14924,7 @@
       <c r="L6" s="122"/>
     </row>
     <row r="7" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A7" s="308"/>
+      <c r="A7" s="310"/>
       <c r="B7" s="135" t="s">
         <v>324</v>
       </c>
@@ -14860,7 +14932,7 @@
         <v>708</v>
       </c>
       <c r="D7" s="253"/>
-      <c r="E7" s="311"/>
+      <c r="E7" s="313"/>
       <c r="F7" s="135" t="s">
         <v>1004</v>
       </c>
@@ -14868,7 +14940,7 @@
         <v>1031</v>
       </c>
       <c r="H7" s="125"/>
-      <c r="I7" s="311"/>
+      <c r="I7" s="313"/>
       <c r="J7" s="135" t="s">
         <v>1094</v>
       </c>
@@ -14878,7 +14950,7 @@
       <c r="L7" s="122"/>
     </row>
     <row r="8" spans="1:12" ht="18.75">
-      <c r="A8" s="306" t="s">
+      <c r="A8" s="308" t="s">
         <v>667</v>
       </c>
       <c r="B8" s="132" t="s">
@@ -14888,7 +14960,7 @@
         <v>709</v>
       </c>
       <c r="D8" s="253"/>
-      <c r="E8" s="309" t="s">
+      <c r="E8" s="311" t="s">
         <v>974</v>
       </c>
       <c r="F8" s="132" t="s">
@@ -14898,7 +14970,7 @@
         <v>1032</v>
       </c>
       <c r="H8" s="125"/>
-      <c r="I8" s="309" t="s">
+      <c r="I8" s="311" t="s">
         <v>1058</v>
       </c>
       <c r="J8" s="132" t="s">
@@ -14910,7 +14982,7 @@
       <c r="L8" s="122"/>
     </row>
     <row r="9" spans="1:12" ht="18.75">
-      <c r="A9" s="307"/>
+      <c r="A9" s="309"/>
       <c r="B9" s="131" t="s">
         <v>658</v>
       </c>
@@ -14918,7 +14990,7 @@
         <v>710</v>
       </c>
       <c r="D9" s="253"/>
-      <c r="E9" s="310"/>
+      <c r="E9" s="312"/>
       <c r="F9" s="131" t="s">
         <v>1006</v>
       </c>
@@ -14926,7 +14998,7 @@
         <v>1033</v>
       </c>
       <c r="H9" s="125"/>
-      <c r="I9" s="310"/>
+      <c r="I9" s="312"/>
       <c r="J9" s="131" t="s">
         <v>1095</v>
       </c>
@@ -14936,7 +15008,7 @@
       <c r="L9" s="122"/>
     </row>
     <row r="10" spans="1:12" ht="18.75">
-      <c r="A10" s="307"/>
+      <c r="A10" s="309"/>
       <c r="B10" s="131" t="s">
         <v>659</v>
       </c>
@@ -14944,7 +15016,7 @@
         <v>711</v>
       </c>
       <c r="D10" s="253"/>
-      <c r="E10" s="310"/>
+      <c r="E10" s="312"/>
       <c r="F10" s="131" t="s">
         <v>1008</v>
       </c>
@@ -14952,7 +15024,7 @@
         <v>1034</v>
       </c>
       <c r="H10" s="125"/>
-      <c r="I10" s="310"/>
+      <c r="I10" s="312"/>
       <c r="J10" s="131" t="s">
         <v>1096</v>
       </c>
@@ -14962,7 +15034,7 @@
       <c r="L10" s="122"/>
     </row>
     <row r="11" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A11" s="308"/>
+      <c r="A11" s="310"/>
       <c r="B11" s="135" t="s">
         <v>660</v>
       </c>
@@ -14970,7 +15042,7 @@
         <v>712</v>
       </c>
       <c r="D11" s="253"/>
-      <c r="E11" s="311"/>
+      <c r="E11" s="313"/>
       <c r="F11" s="135" t="s">
         <v>1009</v>
       </c>
@@ -14978,7 +15050,7 @@
         <v>1035</v>
       </c>
       <c r="H11" s="125"/>
-      <c r="I11" s="311"/>
+      <c r="I11" s="313"/>
       <c r="J11" s="135" t="s">
         <v>1097</v>
       </c>
@@ -14988,7 +15060,7 @@
       <c r="L11" s="122"/>
     </row>
     <row r="12" spans="1:12" ht="18.75">
-      <c r="A12" s="306" t="s">
+      <c r="A12" s="308" t="s">
         <v>665</v>
       </c>
       <c r="B12" s="132" t="s">
@@ -14998,7 +15070,7 @@
         <v>713</v>
       </c>
       <c r="D12" s="253"/>
-      <c r="E12" s="309" t="s">
+      <c r="E12" s="311" t="s">
         <v>973</v>
       </c>
       <c r="F12" s="132" t="s">
@@ -15008,7 +15080,7 @@
         <v>1036</v>
       </c>
       <c r="H12" s="125"/>
-      <c r="I12" s="309" t="s">
+      <c r="I12" s="311" t="s">
         <v>1059</v>
       </c>
       <c r="J12" s="132" t="s">
@@ -15020,7 +15092,7 @@
       <c r="L12" s="122"/>
     </row>
     <row r="13" spans="1:12" ht="18.75">
-      <c r="A13" s="307"/>
+      <c r="A13" s="309"/>
       <c r="B13" s="131" t="s">
         <v>662</v>
       </c>
@@ -15028,7 +15100,7 @@
         <v>714</v>
       </c>
       <c r="D13" s="253"/>
-      <c r="E13" s="310"/>
+      <c r="E13" s="312"/>
       <c r="F13" s="131" t="s">
         <v>1011</v>
       </c>
@@ -15036,7 +15108,7 @@
         <v>1037</v>
       </c>
       <c r="H13" s="125"/>
-      <c r="I13" s="310"/>
+      <c r="I13" s="312"/>
       <c r="J13" s="131" t="s">
         <v>1099</v>
       </c>
@@ -15046,7 +15118,7 @@
       <c r="L13" s="122"/>
     </row>
     <row r="14" spans="1:12" ht="18.75">
-      <c r="A14" s="307"/>
+      <c r="A14" s="309"/>
       <c r="B14" s="131" t="s">
         <v>663</v>
       </c>
@@ -15054,7 +15126,7 @@
         <v>715</v>
       </c>
       <c r="D14" s="253"/>
-      <c r="E14" s="310"/>
+      <c r="E14" s="312"/>
       <c r="F14" s="131" t="s">
         <v>1012</v>
       </c>
@@ -15062,7 +15134,7 @@
         <v>1038</v>
       </c>
       <c r="H14" s="125"/>
-      <c r="I14" s="310"/>
+      <c r="I14" s="312"/>
       <c r="J14" s="131" t="s">
         <v>1100</v>
       </c>
@@ -15072,7 +15144,7 @@
       <c r="L14" s="122"/>
     </row>
     <row r="15" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A15" s="308"/>
+      <c r="A15" s="310"/>
       <c r="B15" s="135" t="s">
         <v>664</v>
       </c>
@@ -15080,7 +15152,7 @@
         <v>716</v>
       </c>
       <c r="D15" s="253"/>
-      <c r="E15" s="311"/>
+      <c r="E15" s="313"/>
       <c r="F15" s="135" t="s">
         <v>1013</v>
       </c>
@@ -15088,7 +15160,7 @@
         <v>1039</v>
       </c>
       <c r="H15" s="125"/>
-      <c r="I15" s="311"/>
+      <c r="I15" s="313"/>
       <c r="J15" s="135" t="s">
         <v>1101</v>
       </c>
@@ -15098,7 +15170,7 @@
       <c r="L15" s="122"/>
     </row>
     <row r="16" spans="1:12" ht="18.75">
-      <c r="A16" s="306" t="s">
+      <c r="A16" s="308" t="s">
         <v>666</v>
       </c>
       <c r="B16" s="132" t="s">
@@ -15108,7 +15180,7 @@
         <v>717</v>
       </c>
       <c r="D16" s="253"/>
-      <c r="E16" s="309" t="s">
+      <c r="E16" s="311" t="s">
         <v>972</v>
       </c>
       <c r="F16" s="132" t="s">
@@ -15118,7 +15190,7 @@
         <v>1040</v>
       </c>
       <c r="H16" s="125"/>
-      <c r="I16" s="309" t="s">
+      <c r="I16" s="311" t="s">
         <v>1060</v>
       </c>
       <c r="J16" s="132" t="s">
@@ -15130,7 +15202,7 @@
       <c r="L16" s="122"/>
     </row>
     <row r="17" spans="1:12" ht="18.75">
-      <c r="A17" s="307"/>
+      <c r="A17" s="309"/>
       <c r="B17" s="131" t="s">
         <v>669</v>
       </c>
@@ -15138,7 +15210,7 @@
         <v>718</v>
       </c>
       <c r="D17" s="253"/>
-      <c r="E17" s="310"/>
+      <c r="E17" s="312"/>
       <c r="F17" s="131" t="s">
         <v>1015</v>
       </c>
@@ -15146,7 +15218,7 @@
         <v>1041</v>
       </c>
       <c r="H17" s="125"/>
-      <c r="I17" s="310"/>
+      <c r="I17" s="312"/>
       <c r="J17" s="131" t="s">
         <v>1103</v>
       </c>
@@ -15156,7 +15228,7 @@
       <c r="L17" s="122"/>
     </row>
     <row r="18" spans="1:12" ht="18.75">
-      <c r="A18" s="307"/>
+      <c r="A18" s="309"/>
       <c r="B18" s="131" t="s">
         <v>670</v>
       </c>
@@ -15164,7 +15236,7 @@
         <v>719</v>
       </c>
       <c r="D18" s="253"/>
-      <c r="E18" s="310"/>
+      <c r="E18" s="312"/>
       <c r="F18" s="131" t="s">
         <v>1016</v>
       </c>
@@ -15172,7 +15244,7 @@
         <v>1042</v>
       </c>
       <c r="H18" s="125"/>
-      <c r="I18" s="310"/>
+      <c r="I18" s="312"/>
       <c r="J18" s="131" t="s">
         <v>1104</v>
       </c>
@@ -15182,7 +15254,7 @@
       <c r="L18" s="122"/>
     </row>
     <row r="19" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A19" s="308"/>
+      <c r="A19" s="310"/>
       <c r="B19" s="135" t="s">
         <v>671</v>
       </c>
@@ -15190,7 +15262,7 @@
         <v>720</v>
       </c>
       <c r="D19" s="253"/>
-      <c r="E19" s="311"/>
+      <c r="E19" s="313"/>
       <c r="F19" s="135" t="s">
         <v>1017</v>
       </c>
@@ -15198,7 +15270,7 @@
         <v>1043</v>
       </c>
       <c r="H19" s="125"/>
-      <c r="I19" s="311"/>
+      <c r="I19" s="313"/>
       <c r="J19" s="135" t="s">
         <v>1105</v>
       </c>
@@ -15212,7 +15284,7 @@
       <c r="B20" s="125"/>
       <c r="C20" s="125"/>
       <c r="D20" s="125"/>
-      <c r="E20" s="309" t="s">
+      <c r="E20" s="311" t="s">
         <v>560</v>
       </c>
       <c r="F20" s="132" t="s">
@@ -15222,7 +15294,7 @@
         <v>1044</v>
       </c>
       <c r="H20" s="125"/>
-      <c r="I20" s="309" t="s">
+      <c r="I20" s="311" t="s">
         <v>1061</v>
       </c>
       <c r="J20" s="132" t="s">
@@ -15238,7 +15310,7 @@
       <c r="B21" s="125"/>
       <c r="C21" s="125"/>
       <c r="D21" s="125"/>
-      <c r="E21" s="310"/>
+      <c r="E21" s="312"/>
       <c r="F21" s="131" t="s">
         <v>1019</v>
       </c>
@@ -15246,7 +15318,7 @@
         <v>1045</v>
       </c>
       <c r="H21" s="125"/>
-      <c r="I21" s="310"/>
+      <c r="I21" s="312"/>
       <c r="J21" s="131" t="s">
         <v>1107</v>
       </c>
@@ -15260,7 +15332,7 @@
       <c r="B22" s="125"/>
       <c r="C22" s="125"/>
       <c r="D22" s="125"/>
-      <c r="E22" s="310"/>
+      <c r="E22" s="312"/>
       <c r="F22" s="131" t="s">
         <v>1020</v>
       </c>
@@ -15268,7 +15340,7 @@
         <v>1046</v>
       </c>
       <c r="H22" s="125"/>
-      <c r="I22" s="310"/>
+      <c r="I22" s="312"/>
       <c r="J22" s="131" t="s">
         <v>1108</v>
       </c>
@@ -15284,7 +15356,7 @@
       <c r="B23" s="256"/>
       <c r="C23" s="257"/>
       <c r="D23" s="125"/>
-      <c r="E23" s="311"/>
+      <c r="E23" s="313"/>
       <c r="F23" s="135" t="s">
         <v>1021</v>
       </c>
@@ -15292,7 +15364,7 @@
         <v>1047</v>
       </c>
       <c r="H23" s="125"/>
-      <c r="I23" s="311"/>
+      <c r="I23" s="313"/>
       <c r="J23" s="135" t="s">
         <v>1109</v>
       </c>
@@ -15312,7 +15384,7 @@
         <v>321</v>
       </c>
       <c r="D24" s="125"/>
-      <c r="E24" s="309" t="s">
+      <c r="E24" s="311" t="s">
         <v>749</v>
       </c>
       <c r="F24" s="132" t="s">
@@ -15322,7 +15394,7 @@
         <v>1048</v>
       </c>
       <c r="H24" s="125"/>
-      <c r="I24" s="309" t="s">
+      <c r="I24" s="311" t="s">
         <v>1062</v>
       </c>
       <c r="J24" s="132" t="s">
@@ -15334,7 +15406,7 @@
       <c r="L24" s="122"/>
     </row>
     <row r="25" spans="1:12" ht="18.75">
-      <c r="A25" s="303" t="s">
+      <c r="A25" s="305" t="s">
         <v>493</v>
       </c>
       <c r="B25" s="132" t="s">
@@ -15344,7 +15416,7 @@
         <v>721</v>
       </c>
       <c r="D25" s="125"/>
-      <c r="E25" s="310"/>
+      <c r="E25" s="312"/>
       <c r="F25" s="131" t="s">
         <v>1023</v>
       </c>
@@ -15352,7 +15424,7 @@
         <v>1049</v>
       </c>
       <c r="H25" s="125"/>
-      <c r="I25" s="310"/>
+      <c r="I25" s="312"/>
       <c r="J25" s="131" t="s">
         <v>1111</v>
       </c>
@@ -15362,7 +15434,7 @@
       <c r="L25" s="122"/>
     </row>
     <row r="26" spans="1:12" ht="18.75">
-      <c r="A26" s="304"/>
+      <c r="A26" s="306"/>
       <c r="B26" s="131" t="s">
         <v>679</v>
       </c>
@@ -15370,7 +15442,7 @@
         <v>722</v>
       </c>
       <c r="D26" s="125"/>
-      <c r="E26" s="310"/>
+      <c r="E26" s="312"/>
       <c r="F26" s="131" t="s">
         <v>1024</v>
       </c>
@@ -15378,7 +15450,7 @@
         <v>1050</v>
       </c>
       <c r="H26" s="125"/>
-      <c r="I26" s="310"/>
+      <c r="I26" s="312"/>
       <c r="J26" s="131" t="s">
         <v>1112</v>
       </c>
@@ -15388,7 +15460,7 @@
       <c r="L26" s="122"/>
     </row>
     <row r="27" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A27" s="304"/>
+      <c r="A27" s="306"/>
       <c r="B27" s="131" t="s">
         <v>680</v>
       </c>
@@ -15396,7 +15468,7 @@
         <v>723</v>
       </c>
       <c r="D27" s="125"/>
-      <c r="E27" s="311"/>
+      <c r="E27" s="313"/>
       <c r="F27" s="135" t="s">
         <v>1025</v>
       </c>
@@ -15404,7 +15476,7 @@
         <v>1051</v>
       </c>
       <c r="H27" s="125"/>
-      <c r="I27" s="311"/>
+      <c r="I27" s="313"/>
       <c r="J27" s="135" t="s">
         <v>1113</v>
       </c>
@@ -15414,7 +15486,7 @@
       <c r="L27" s="122"/>
     </row>
     <row r="28" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A28" s="305"/>
+      <c r="A28" s="307"/>
       <c r="B28" s="135" t="s">
         <v>681</v>
       </c>
@@ -15422,7 +15494,7 @@
         <v>724</v>
       </c>
       <c r="D28" s="125"/>
-      <c r="E28" s="309" t="s">
+      <c r="E28" s="311" t="s">
         <v>562</v>
       </c>
       <c r="F28" s="132" t="s">
@@ -15432,7 +15504,7 @@
         <v>1052</v>
       </c>
       <c r="H28" s="125"/>
-      <c r="I28" s="309" t="s">
+      <c r="I28" s="311" t="s">
         <v>1063</v>
       </c>
       <c r="J28" s="132" t="s">
@@ -15444,7 +15516,7 @@
       <c r="L28" s="122"/>
     </row>
     <row r="29" spans="1:12" ht="18.75">
-      <c r="A29" s="303" t="s">
+      <c r="A29" s="305" t="s">
         <v>687</v>
       </c>
       <c r="B29" s="132" t="s">
@@ -15454,7 +15526,7 @@
         <v>725</v>
       </c>
       <c r="D29" s="253"/>
-      <c r="E29" s="310"/>
+      <c r="E29" s="312"/>
       <c r="F29" s="131" t="s">
         <v>1027</v>
       </c>
@@ -15462,7 +15534,7 @@
         <v>1053</v>
       </c>
       <c r="H29" s="125"/>
-      <c r="I29" s="310"/>
+      <c r="I29" s="312"/>
       <c r="J29" s="131" t="s">
         <v>1115</v>
       </c>
@@ -15472,7 +15544,7 @@
       <c r="L29" s="122"/>
     </row>
     <row r="30" spans="1:12" ht="18.75">
-      <c r="A30" s="304"/>
+      <c r="A30" s="306"/>
       <c r="B30" s="131" t="s">
         <v>684</v>
       </c>
@@ -15480,11 +15552,11 @@
         <v>726</v>
       </c>
       <c r="D30" s="253"/>
-      <c r="E30" s="310"/>
+      <c r="E30" s="312"/>
       <c r="F30" s="131"/>
       <c r="G30" s="250"/>
       <c r="H30" s="125"/>
-      <c r="I30" s="310"/>
+      <c r="I30" s="312"/>
       <c r="J30" s="131" t="s">
         <v>1116</v>
       </c>
@@ -15494,7 +15566,7 @@
       <c r="L30" s="122"/>
     </row>
     <row r="31" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A31" s="304"/>
+      <c r="A31" s="306"/>
       <c r="B31" s="131" t="s">
         <v>685</v>
       </c>
@@ -15502,11 +15574,11 @@
         <v>727</v>
       </c>
       <c r="D31" s="253"/>
-      <c r="E31" s="311"/>
+      <c r="E31" s="313"/>
       <c r="F31" s="135"/>
       <c r="G31" s="251"/>
       <c r="H31" s="125"/>
-      <c r="I31" s="311"/>
+      <c r="I31" s="313"/>
       <c r="J31" s="135" t="s">
         <v>1117</v>
       </c>
@@ -15516,7 +15588,7 @@
       <c r="L31" s="122"/>
     </row>
     <row r="32" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A32" s="305"/>
+      <c r="A32" s="307"/>
       <c r="B32" s="135" t="s">
         <v>686</v>
       </c>
@@ -15534,7 +15606,7 @@
       <c r="L32" s="122"/>
     </row>
     <row r="33" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A33" s="303" t="s">
+      <c r="A33" s="305" t="s">
         <v>691</v>
       </c>
       <c r="B33" s="132" t="s">
@@ -15544,21 +15616,21 @@
         <v>729</v>
       </c>
       <c r="D33" s="253"/>
-      <c r="E33" s="318" t="s">
+      <c r="E33" s="320" t="s">
         <v>1148</v>
       </c>
-      <c r="F33" s="319"/>
-      <c r="G33" s="320"/>
+      <c r="F33" s="321"/>
+      <c r="G33" s="322"/>
       <c r="H33" s="124"/>
-      <c r="I33" s="318" t="s">
+      <c r="I33" s="320" t="s">
         <v>1147</v>
       </c>
-      <c r="J33" s="319"/>
-      <c r="K33" s="320"/>
+      <c r="J33" s="321"/>
+      <c r="K33" s="322"/>
       <c r="L33" s="122"/>
     </row>
     <row r="34" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A34" s="304"/>
+      <c r="A34" s="306"/>
       <c r="B34" s="131" t="s">
         <v>693</v>
       </c>
@@ -15588,7 +15660,7 @@
       <c r="L34" s="122"/>
     </row>
     <row r="35" spans="1:12" ht="18.75">
-      <c r="A35" s="304"/>
+      <c r="A35" s="306"/>
       <c r="B35" s="131" t="s">
         <v>694</v>
       </c>
@@ -15596,7 +15668,7 @@
         <v>731</v>
       </c>
       <c r="D35" s="253"/>
-      <c r="E35" s="303" t="s">
+      <c r="E35" s="305" t="s">
         <v>494</v>
       </c>
       <c r="F35" s="132" t="s">
@@ -15606,7 +15678,7 @@
         <v>11311</v>
       </c>
       <c r="H35" s="124"/>
-      <c r="I35" s="303" t="s">
+      <c r="I35" s="305" t="s">
         <v>955</v>
       </c>
       <c r="J35" s="132" t="s">
@@ -15618,7 +15690,7 @@
       <c r="L35" s="122"/>
     </row>
     <row r="36" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A36" s="305"/>
+      <c r="A36" s="307"/>
       <c r="B36" s="135" t="s">
         <v>695</v>
       </c>
@@ -15626,7 +15698,7 @@
         <v>732</v>
       </c>
       <c r="D36" s="253"/>
-      <c r="E36" s="304"/>
+      <c r="E36" s="306"/>
       <c r="F36" s="131" t="s">
         <v>958</v>
       </c>
@@ -15634,7 +15706,7 @@
         <v>11312</v>
       </c>
       <c r="H36" s="124"/>
-      <c r="I36" s="304"/>
+      <c r="I36" s="306"/>
       <c r="J36" s="131" t="s">
         <v>965</v>
       </c>
@@ -15644,7 +15716,7 @@
       <c r="L36" s="122"/>
     </row>
     <row r="37" spans="1:12" ht="18.75">
-      <c r="A37" s="303" t="s">
+      <c r="A37" s="305" t="s">
         <v>698</v>
       </c>
       <c r="B37" s="132" t="s">
@@ -15654,7 +15726,7 @@
         <v>11441</v>
       </c>
       <c r="D37" s="253"/>
-      <c r="E37" s="304"/>
+      <c r="E37" s="306"/>
       <c r="F37" s="131" t="s">
         <v>959</v>
       </c>
@@ -15662,7 +15734,7 @@
         <v>11313</v>
       </c>
       <c r="H37" s="124"/>
-      <c r="I37" s="304"/>
+      <c r="I37" s="306"/>
       <c r="J37" s="131" t="s">
         <v>966</v>
       </c>
@@ -15672,7 +15744,7 @@
       <c r="L37" s="122"/>
     </row>
     <row r="38" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A38" s="304"/>
+      <c r="A38" s="306"/>
       <c r="B38" s="131" t="s">
         <v>700</v>
       </c>
@@ -15680,7 +15752,7 @@
         <v>11442</v>
       </c>
       <c r="D38" s="253"/>
-      <c r="E38" s="305"/>
+      <c r="E38" s="307"/>
       <c r="F38" s="135" t="s">
         <v>959</v>
       </c>
@@ -15688,7 +15760,7 @@
         <v>11314</v>
       </c>
       <c r="H38" s="124"/>
-      <c r="I38" s="305"/>
+      <c r="I38" s="307"/>
       <c r="J38" s="135" t="s">
         <v>967</v>
       </c>
@@ -15698,7 +15770,7 @@
       <c r="L38" s="122"/>
     </row>
     <row r="39" spans="1:12" ht="18.75">
-      <c r="A39" s="304"/>
+      <c r="A39" s="306"/>
       <c r="B39" s="131" t="s">
         <v>701</v>
       </c>
@@ -15706,7 +15778,7 @@
         <v>11443</v>
       </c>
       <c r="D39" s="253"/>
-      <c r="E39" s="303" t="s">
+      <c r="E39" s="305" t="s">
         <v>954</v>
       </c>
       <c r="F39" s="132" t="s">
@@ -15716,7 +15788,7 @@
         <v>11321</v>
       </c>
       <c r="H39" s="124"/>
-      <c r="I39" s="303" t="s">
+      <c r="I39" s="305" t="s">
         <v>956</v>
       </c>
       <c r="J39" s="132" t="s">
@@ -15728,7 +15800,7 @@
       <c r="L39" s="122"/>
     </row>
     <row r="40" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A40" s="305"/>
+      <c r="A40" s="307"/>
       <c r="B40" s="135" t="s">
         <v>702</v>
       </c>
@@ -15736,7 +15808,7 @@
         <v>11444</v>
       </c>
       <c r="D40" s="253"/>
-      <c r="E40" s="304"/>
+      <c r="E40" s="306"/>
       <c r="F40" s="131" t="s">
         <v>961</v>
       </c>
@@ -15744,7 +15816,7 @@
         <v>11322</v>
       </c>
       <c r="H40" s="124"/>
-      <c r="I40" s="304"/>
+      <c r="I40" s="306"/>
       <c r="J40" s="131" t="s">
         <v>969</v>
       </c>
@@ -15754,7 +15826,7 @@
       <c r="L40" s="122"/>
     </row>
     <row r="41" spans="1:12" ht="18.75">
-      <c r="A41" s="303" t="s">
+      <c r="A41" s="305" t="s">
         <v>1346</v>
       </c>
       <c r="B41" s="132" t="s">
@@ -15764,7 +15836,7 @@
         <v>11451</v>
       </c>
       <c r="D41" s="253"/>
-      <c r="E41" s="304"/>
+      <c r="E41" s="306"/>
       <c r="F41" s="131" t="s">
         <v>962</v>
       </c>
@@ -15772,7 +15844,7 @@
         <v>11323</v>
       </c>
       <c r="H41" s="124"/>
-      <c r="I41" s="304"/>
+      <c r="I41" s="306"/>
       <c r="J41" s="131" t="s">
         <v>970</v>
       </c>
@@ -15782,7 +15854,7 @@
       <c r="L41" s="122"/>
     </row>
     <row r="42" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A42" s="304"/>
+      <c r="A42" s="306"/>
       <c r="B42" s="131" t="s">
         <v>1348</v>
       </c>
@@ -15790,7 +15862,7 @@
         <v>11452</v>
       </c>
       <c r="D42" s="253"/>
-      <c r="E42" s="305"/>
+      <c r="E42" s="307"/>
       <c r="F42" s="135" t="s">
         <v>963</v>
       </c>
@@ -15798,7 +15870,7 @@
         <v>11324</v>
       </c>
       <c r="H42" s="124"/>
-      <c r="I42" s="305"/>
+      <c r="I42" s="307"/>
       <c r="J42" s="135" t="s">
         <v>971</v>
       </c>
@@ -15808,7 +15880,7 @@
       <c r="L42" s="122"/>
     </row>
     <row r="43" spans="1:12" ht="18.75">
-      <c r="A43" s="304"/>
+      <c r="A43" s="306"/>
       <c r="B43" s="131" t="s">
         <v>1349</v>
       </c>
@@ -15826,7 +15898,7 @@
       <c r="L43" s="122"/>
     </row>
     <row r="44" spans="1:12" ht="19.5" thickBot="1">
-      <c r="A44" s="305"/>
+      <c r="A44" s="307"/>
       <c r="B44" s="135" t="s">
         <v>1350</v>
       </c>
@@ -15917,40 +15989,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="325" t="s">
+      <c r="A1" s="327" t="s">
         <v>1150</v>
       </c>
-      <c r="B1" s="326"/>
-      <c r="C1" s="326"/>
-      <c r="D1" s="326"/>
-      <c r="E1" s="326"/>
-      <c r="F1" s="326"/>
-      <c r="G1" s="326"/>
-      <c r="H1" s="327"/>
+      <c r="B1" s="328"/>
+      <c r="C1" s="328"/>
+      <c r="D1" s="328"/>
+      <c r="E1" s="328"/>
+      <c r="F1" s="328"/>
+      <c r="G1" s="328"/>
+      <c r="H1" s="329"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="328"/>
-      <c r="B2" s="329"/>
-      <c r="C2" s="329"/>
-      <c r="D2" s="329"/>
-      <c r="E2" s="329"/>
-      <c r="F2" s="329"/>
-      <c r="G2" s="329"/>
-      <c r="H2" s="330"/>
+      <c r="A2" s="330"/>
+      <c r="B2" s="331"/>
+      <c r="C2" s="331"/>
+      <c r="D2" s="331"/>
+      <c r="E2" s="331"/>
+      <c r="F2" s="331"/>
+      <c r="G2" s="331"/>
+      <c r="H2" s="332"/>
     </row>
     <row r="3" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A3" s="331" t="s">
+      <c r="A3" s="333" t="s">
         <v>250</v>
       </c>
-      <c r="B3" s="332"/>
-      <c r="C3" s="332"/>
-      <c r="D3" s="332"/>
-      <c r="E3" s="332" t="s">
+      <c r="B3" s="334"/>
+      <c r="C3" s="334"/>
+      <c r="D3" s="334"/>
+      <c r="E3" s="334" t="s">
         <v>251</v>
       </c>
-      <c r="F3" s="332"/>
-      <c r="G3" s="332"/>
-      <c r="H3" s="333"/>
+      <c r="F3" s="334"/>
+      <c r="G3" s="334"/>
+      <c r="H3" s="335"/>
     </row>
     <row r="4" spans="1:8" ht="18.75" thickBot="1">
       <c r="A4" s="12">
@@ -16484,11 +16556,11 @@
       <c r="C27" s="118" t="s">
         <v>594</v>
       </c>
-      <c r="D27" s="324" t="s">
+      <c r="D27" s="326" t="s">
         <v>570</v>
       </c>
-      <c r="E27" s="324"/>
-      <c r="F27" s="324"/>
+      <c r="E27" s="326"/>
+      <c r="F27" s="326"/>
       <c r="G27" s="17"/>
       <c r="H27" s="18"/>
     </row>
@@ -16500,11 +16572,11 @@
       <c r="C28" s="118" t="s">
         <v>598</v>
       </c>
-      <c r="D28" s="324" t="s">
+      <c r="D28" s="326" t="s">
         <v>4</v>
       </c>
-      <c r="E28" s="324"/>
-      <c r="F28" s="324"/>
+      <c r="E28" s="326"/>
+      <c r="F28" s="326"/>
       <c r="G28" s="17"/>
       <c r="H28" s="18"/>
     </row>
@@ -16516,11 +16588,11 @@
       <c r="C29" s="118" t="s">
         <v>599</v>
       </c>
-      <c r="D29" s="324" t="s">
+      <c r="D29" s="326" t="s">
         <v>571</v>
       </c>
-      <c r="E29" s="324"/>
-      <c r="F29" s="324"/>
+      <c r="E29" s="326"/>
+      <c r="F29" s="326"/>
       <c r="G29" s="17"/>
       <c r="H29" s="18"/>
     </row>
@@ -16532,11 +16604,11 @@
       <c r="C30" s="118" t="s">
         <v>600</v>
       </c>
-      <c r="D30" s="324" t="s">
+      <c r="D30" s="326" t="s">
         <v>572</v>
       </c>
-      <c r="E30" s="324"/>
-      <c r="F30" s="324"/>
+      <c r="E30" s="326"/>
+      <c r="F30" s="326"/>
       <c r="G30" s="17"/>
       <c r="H30" s="18"/>
     </row>
@@ -16548,11 +16620,11 @@
       <c r="C31" s="118" t="s">
         <v>601</v>
       </c>
-      <c r="D31" s="324" t="s">
+      <c r="D31" s="326" t="s">
         <v>573</v>
       </c>
-      <c r="E31" s="324"/>
-      <c r="F31" s="324"/>
+      <c r="E31" s="326"/>
+      <c r="F31" s="326"/>
       <c r="G31" s="17"/>
       <c r="H31" s="18"/>
     </row>
@@ -16564,11 +16636,11 @@
       <c r="C32" s="118" t="s">
         <v>602</v>
       </c>
-      <c r="D32" s="324" t="s">
+      <c r="D32" s="326" t="s">
         <v>574</v>
       </c>
-      <c r="E32" s="324"/>
-      <c r="F32" s="324"/>
+      <c r="E32" s="326"/>
+      <c r="F32" s="326"/>
       <c r="G32" s="17"/>
       <c r="H32" s="18"/>
     </row>
@@ -16580,11 +16652,11 @@
       <c r="C33" s="118" t="s">
         <v>614</v>
       </c>
-      <c r="D33" s="324" t="s">
+      <c r="D33" s="326" t="s">
         <v>482</v>
       </c>
-      <c r="E33" s="324"/>
-      <c r="F33" s="324"/>
+      <c r="E33" s="326"/>
+      <c r="F33" s="326"/>
       <c r="G33" s="17"/>
       <c r="H33" s="18"/>
     </row>
@@ -16596,11 +16668,11 @@
       <c r="C34" s="118" t="s">
         <v>615</v>
       </c>
-      <c r="D34" s="324" t="s">
+      <c r="D34" s="326" t="s">
         <v>575</v>
       </c>
-      <c r="E34" s="324"/>
-      <c r="F34" s="324"/>
+      <c r="E34" s="326"/>
+      <c r="F34" s="326"/>
       <c r="G34" s="17"/>
       <c r="H34" s="18"/>
     </row>
@@ -16612,11 +16684,11 @@
       <c r="C35" s="118" t="s">
         <v>616</v>
       </c>
-      <c r="D35" s="324" t="s">
+      <c r="D35" s="326" t="s">
         <v>576</v>
       </c>
-      <c r="E35" s="324"/>
-      <c r="F35" s="324"/>
+      <c r="E35" s="326"/>
+      <c r="F35" s="326"/>
       <c r="G35" s="17"/>
       <c r="H35" s="18"/>
     </row>
@@ -16626,11 +16698,11 @@
       <c r="C36" s="118" t="s">
         <v>651</v>
       </c>
-      <c r="D36" s="321" t="s">
+      <c r="D36" s="323" t="s">
         <v>591</v>
       </c>
-      <c r="E36" s="322"/>
-      <c r="F36" s="323"/>
+      <c r="E36" s="324"/>
+      <c r="F36" s="325"/>
       <c r="G36" s="17"/>
       <c r="H36" s="18"/>
     </row>
@@ -16640,11 +16712,11 @@
       <c r="C37" s="118" t="s">
         <v>654</v>
       </c>
-      <c r="D37" s="321" t="s">
+      <c r="D37" s="323" t="s">
         <v>652</v>
       </c>
-      <c r="E37" s="322"/>
-      <c r="F37" s="323"/>
+      <c r="E37" s="324"/>
+      <c r="F37" s="325"/>
       <c r="G37" s="17"/>
       <c r="H37" s="18"/>
     </row>
@@ -16654,11 +16726,11 @@
       <c r="C38" s="118" t="s">
         <v>653</v>
       </c>
-      <c r="D38" s="321" t="s">
+      <c r="D38" s="323" t="s">
         <v>655</v>
       </c>
-      <c r="E38" s="322"/>
-      <c r="F38" s="323"/>
+      <c r="E38" s="324"/>
+      <c r="F38" s="325"/>
       <c r="G38" s="17"/>
       <c r="H38" s="18"/>
     </row>
@@ -16666,9 +16738,9 @@
       <c r="A39" s="16"/>
       <c r="B39" s="120"/>
       <c r="C39" s="118"/>
-      <c r="D39" s="321"/>
-      <c r="E39" s="322"/>
-      <c r="F39" s="323"/>
+      <c r="D39" s="323"/>
+      <c r="E39" s="324"/>
+      <c r="F39" s="325"/>
       <c r="G39" s="17"/>
       <c r="H39" s="18"/>
     </row>
@@ -16804,28 +16876,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75">
-      <c r="A1" s="343" t="s">
+      <c r="A1" s="345" t="s">
         <v>1183</v>
       </c>
-      <c r="B1" s="343"/>
-      <c r="C1" s="343"/>
-      <c r="D1" s="343"/>
-      <c r="E1" s="343"/>
-      <c r="F1" s="343"/>
-      <c r="G1" s="343"/>
-      <c r="H1" s="343"/>
+      <c r="B1" s="345"/>
+      <c r="C1" s="345"/>
+      <c r="D1" s="345"/>
+      <c r="E1" s="345"/>
+      <c r="F1" s="345"/>
+      <c r="G1" s="345"/>
+      <c r="H1" s="345"/>
     </row>
     <row r="2" spans="1:10" ht="15.75">
-      <c r="A2" s="337" t="s">
+      <c r="A2" s="339" t="s">
         <v>1151</v>
       </c>
-      <c r="B2" s="338"/>
-      <c r="C2" s="338"/>
-      <c r="D2" s="338"/>
-      <c r="E2" s="338"/>
-      <c r="F2" s="338"/>
-      <c r="G2" s="338"/>
-      <c r="H2" s="339"/>
+      <c r="B2" s="340"/>
+      <c r="C2" s="340"/>
+      <c r="D2" s="340"/>
+      <c r="E2" s="340"/>
+      <c r="F2" s="340"/>
+      <c r="G2" s="340"/>
+      <c r="H2" s="341"/>
     </row>
     <row r="3" spans="1:10" ht="15.75">
       <c r="A3" s="5"/>
@@ -17141,16 +17213,16 @@
       <c r="H17" s="263"/>
     </row>
     <row r="18" spans="1:11" ht="15.75">
-      <c r="A18" s="340" t="s">
+      <c r="A18" s="342" t="s">
         <v>224</v>
       </c>
-      <c r="B18" s="341"/>
-      <c r="C18" s="341"/>
-      <c r="D18" s="341"/>
-      <c r="E18" s="341"/>
-      <c r="F18" s="341"/>
-      <c r="G18" s="341"/>
-      <c r="H18" s="342"/>
+      <c r="B18" s="343"/>
+      <c r="C18" s="343"/>
+      <c r="D18" s="343"/>
+      <c r="E18" s="343"/>
+      <c r="F18" s="343"/>
+      <c r="G18" s="343"/>
+      <c r="H18" s="344"/>
     </row>
     <row r="19" spans="1:11" ht="15.75">
       <c r="A19" s="264"/>
@@ -17406,16 +17478,16 @@
       <c r="H30" s="4"/>
     </row>
     <row r="31" spans="1:11" ht="15.75">
-      <c r="A31" s="337" t="s">
+      <c r="A31" s="339" t="s">
         <v>225</v>
       </c>
-      <c r="B31" s="338"/>
-      <c r="C31" s="338"/>
-      <c r="D31" s="338"/>
-      <c r="E31" s="338"/>
-      <c r="F31" s="338"/>
-      <c r="G31" s="338"/>
-      <c r="H31" s="339"/>
+      <c r="B31" s="340"/>
+      <c r="C31" s="340"/>
+      <c r="D31" s="340"/>
+      <c r="E31" s="340"/>
+      <c r="F31" s="340"/>
+      <c r="G31" s="340"/>
+      <c r="H31" s="341"/>
     </row>
     <row r="32" spans="1:11" ht="15.75">
       <c r="A32" s="5"/>
@@ -17641,18 +17713,18 @@
     </row>
     <row r="43" spans="1:8" ht="10.5" customHeight="1"/>
     <row r="44" spans="1:8" ht="15.75">
-      <c r="A44" s="334" t="s">
+      <c r="A44" s="336" t="s">
         <v>1174</v>
       </c>
-      <c r="B44" s="335"/>
-      <c r="C44" s="335"/>
-      <c r="D44" s="336"/>
-      <c r="E44" s="334" t="s">
+      <c r="B44" s="337"/>
+      <c r="C44" s="337"/>
+      <c r="D44" s="338"/>
+      <c r="E44" s="336" t="s">
         <v>1174</v>
       </c>
-      <c r="F44" s="335"/>
-      <c r="G44" s="335"/>
-      <c r="H44" s="336"/>
+      <c r="F44" s="337"/>
+      <c r="G44" s="337"/>
+      <c r="H44" s="338"/>
     </row>
     <row r="45" spans="1:8" ht="15.75">
       <c r="A45" s="3"/>
@@ -17765,54 +17837,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="14.45" customHeight="1">
-      <c r="A1" s="347" t="s">
+      <c r="A1" s="349" t="s">
         <v>1295</v>
       </c>
-      <c r="B1" s="348"/>
-      <c r="C1" s="348"/>
-      <c r="D1" s="348"/>
-      <c r="E1" s="348"/>
-      <c r="F1" s="348"/>
-      <c r="G1" s="348"/>
-      <c r="H1" s="349"/>
+      <c r="B1" s="350"/>
+      <c r="C1" s="350"/>
+      <c r="D1" s="350"/>
+      <c r="E1" s="350"/>
+      <c r="F1" s="350"/>
+      <c r="G1" s="350"/>
+      <c r="H1" s="351"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1">
-      <c r="A2" s="350"/>
-      <c r="B2" s="351"/>
-      <c r="C2" s="351"/>
-      <c r="D2" s="351"/>
-      <c r="E2" s="351"/>
-      <c r="F2" s="351"/>
-      <c r="G2" s="351"/>
-      <c r="H2" s="352"/>
+      <c r="A2" s="352"/>
+      <c r="B2" s="353"/>
+      <c r="C2" s="353"/>
+      <c r="D2" s="353"/>
+      <c r="E2" s="353"/>
+      <c r="F2" s="353"/>
+      <c r="G2" s="353"/>
+      <c r="H2" s="354"/>
     </row>
     <row r="3" spans="1:8" ht="23.25">
-      <c r="A3" s="353" t="s">
+      <c r="A3" s="355" t="s">
         <v>1255</v>
       </c>
-      <c r="B3" s="354"/>
-      <c r="C3" s="354"/>
-      <c r="D3" s="355"/>
-      <c r="E3" s="356" t="s">
+      <c r="B3" s="356"/>
+      <c r="C3" s="356"/>
+      <c r="D3" s="357"/>
+      <c r="E3" s="358" t="s">
         <v>1256</v>
       </c>
-      <c r="F3" s="354"/>
-      <c r="G3" s="354"/>
-      <c r="H3" s="357"/>
+      <c r="F3" s="356"/>
+      <c r="G3" s="356"/>
+      <c r="H3" s="359"/>
     </row>
     <row r="4" spans="1:8" ht="16.149999999999999" customHeight="1" thickBot="1">
-      <c r="A4" s="358" t="s">
+      <c r="A4" s="360" t="s">
         <v>1257</v>
       </c>
-      <c r="B4" s="359"/>
-      <c r="C4" s="359"/>
-      <c r="D4" s="360"/>
-      <c r="E4" s="361" t="s">
+      <c r="B4" s="361"/>
+      <c r="C4" s="361"/>
+      <c r="D4" s="362"/>
+      <c r="E4" s="363" t="s">
         <v>1258</v>
       </c>
-      <c r="F4" s="359"/>
-      <c r="G4" s="359"/>
-      <c r="H4" s="362"/>
+      <c r="F4" s="361"/>
+      <c r="G4" s="361"/>
+      <c r="H4" s="364"/>
     </row>
     <row r="5" spans="1:8" ht="19.5" thickBot="1">
       <c r="A5" s="272">
@@ -18291,12 +18363,12 @@
       </c>
     </row>
     <row r="25" spans="1:8" ht="19.5" thickBot="1">
-      <c r="A25" s="344" t="s">
+      <c r="A25" s="346" t="s">
         <v>1287</v>
       </c>
-      <c r="B25" s="345"/>
-      <c r="C25" s="345"/>
-      <c r="D25" s="346"/>
+      <c r="B25" s="347"/>
+      <c r="C25" s="347"/>
+      <c r="D25" s="348"/>
       <c r="E25" s="273">
         <v>21</v>
       </c>
@@ -18529,28 +18601,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="20.100000000000001" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A1" s="363" t="s">
+      <c r="A1" s="365" t="s">
         <v>952</v>
       </c>
-      <c r="B1" s="364"/>
-      <c r="C1" s="364"/>
-      <c r="D1" s="364"/>
-      <c r="E1" s="364"/>
-      <c r="F1" s="365"/>
+      <c r="B1" s="366"/>
+      <c r="C1" s="366"/>
+      <c r="D1" s="366"/>
+      <c r="E1" s="366"/>
+      <c r="F1" s="367"/>
       <c r="G1" s="175"/>
       <c r="H1" s="175"/>
     </row>
     <row r="2" spans="1:8" ht="20.100000000000001" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A2" s="366" t="s">
+      <c r="A2" s="368" t="s">
         <v>840</v>
       </c>
-      <c r="B2" s="367"/>
-      <c r="C2" s="368"/>
-      <c r="D2" s="366" t="s">
+      <c r="B2" s="369"/>
+      <c r="C2" s="370"/>
+      <c r="D2" s="368" t="s">
         <v>841</v>
       </c>
-      <c r="E2" s="367"/>
-      <c r="F2" s="368"/>
+      <c r="E2" s="369"/>
+      <c r="F2" s="370"/>
       <c r="G2" s="175"/>
       <c r="H2" s="175"/>
     </row>
@@ -18574,7 +18646,7 @@
         <v>1</v>
       </c>
       <c r="G3" s="175"/>
-      <c r="H3" s="369" t="s">
+      <c r="H3" s="371" t="s">
         <v>844</v>
       </c>
     </row>
@@ -18598,7 +18670,7 @@
         <v>2</v>
       </c>
       <c r="G4" s="175"/>
-      <c r="H4" s="370"/>
+      <c r="H4" s="372"/>
     </row>
     <row r="5" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A5" s="176">
@@ -18620,7 +18692,7 @@
         <v>3</v>
       </c>
       <c r="G5" s="175"/>
-      <c r="H5" s="370"/>
+      <c r="H5" s="372"/>
     </row>
     <row r="6" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A6" s="179">
@@ -18642,7 +18714,7 @@
         <v>4</v>
       </c>
       <c r="G6" s="175"/>
-      <c r="H6" s="370"/>
+      <c r="H6" s="372"/>
     </row>
     <row r="7" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A7" s="179">
@@ -18664,7 +18736,7 @@
         <v>5</v>
       </c>
       <c r="G7" s="175"/>
-      <c r="H7" s="370"/>
+      <c r="H7" s="372"/>
     </row>
     <row r="8" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A8" s="182">
@@ -18686,7 +18758,7 @@
         <v>6</v>
       </c>
       <c r="G8" s="175"/>
-      <c r="H8" s="370"/>
+      <c r="H8" s="372"/>
     </row>
     <row r="9" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A9" s="182">
@@ -18708,7 +18780,7 @@
         <v>7</v>
       </c>
       <c r="G9" s="175"/>
-      <c r="H9" s="370"/>
+      <c r="H9" s="372"/>
     </row>
     <row r="10" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A10" s="185">
@@ -18730,7 +18802,7 @@
         <v>8</v>
       </c>
       <c r="G10" s="175"/>
-      <c r="H10" s="371"/>
+      <c r="H10" s="373"/>
     </row>
     <row r="11" spans="1:8" ht="20.100000000000001" customHeight="1" thickTop="1" thickBot="1">
       <c r="A11" s="188">
@@ -18752,7 +18824,7 @@
         <v>9</v>
       </c>
       <c r="G11" s="175"/>
-      <c r="H11" s="372" t="s">
+      <c r="H11" s="374" t="s">
         <v>856</v>
       </c>
     </row>
@@ -18776,7 +18848,7 @@
         <v>10</v>
       </c>
       <c r="G12" s="175"/>
-      <c r="H12" s="373"/>
+      <c r="H12" s="375"/>
     </row>
     <row r="13" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A13" s="191">
@@ -18798,7 +18870,7 @@
         <v>11</v>
       </c>
       <c r="G13" s="175"/>
-      <c r="H13" s="373"/>
+      <c r="H13" s="375"/>
     </row>
     <row r="14" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A14" s="191">
@@ -18820,7 +18892,7 @@
         <v>12</v>
       </c>
       <c r="G14" s="175"/>
-      <c r="H14" s="373"/>
+      <c r="H14" s="375"/>
     </row>
     <row r="15" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A15" s="195">
@@ -18842,7 +18914,7 @@
         <v>13</v>
       </c>
       <c r="G15" s="175"/>
-      <c r="H15" s="373"/>
+      <c r="H15" s="375"/>
     </row>
     <row r="16" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A16" s="195">
@@ -18864,7 +18936,7 @@
         <v>14</v>
       </c>
       <c r="G16" s="175"/>
-      <c r="H16" s="373"/>
+      <c r="H16" s="375"/>
     </row>
     <row r="17" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A17" s="195">
@@ -18886,7 +18958,7 @@
         <v>15</v>
       </c>
       <c r="G17" s="175"/>
-      <c r="H17" s="373"/>
+      <c r="H17" s="375"/>
     </row>
     <row r="18" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A18" s="195">
@@ -18908,7 +18980,7 @@
         <v>16</v>
       </c>
       <c r="G18" s="175"/>
-      <c r="H18" s="373"/>
+      <c r="H18" s="375"/>
     </row>
     <row r="19" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A19" s="195">
@@ -18930,7 +19002,7 @@
         <v>17</v>
       </c>
       <c r="G19" s="175"/>
-      <c r="H19" s="373"/>
+      <c r="H19" s="375"/>
     </row>
     <row r="20" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A20" s="198">
@@ -18952,7 +19024,7 @@
         <v>18</v>
       </c>
       <c r="G20" s="175"/>
-      <c r="H20" s="373"/>
+      <c r="H20" s="375"/>
     </row>
     <row r="21" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A21" s="198">
@@ -18974,7 +19046,7 @@
         <v>19</v>
       </c>
       <c r="G21" s="175"/>
-      <c r="H21" s="373"/>
+      <c r="H21" s="375"/>
     </row>
     <row r="22" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A22" s="201">
@@ -18996,7 +19068,7 @@
         <v>20</v>
       </c>
       <c r="G22" s="175"/>
-      <c r="H22" s="374"/>
+      <c r="H22" s="376"/>
     </row>
     <row r="23" spans="1:8" ht="20.100000000000001" customHeight="1" thickTop="1"/>
     <row r="24" spans="1:8" ht="20.100000000000001" customHeight="1"/>
@@ -19014,28 +19086,28 @@
     <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1"/>
     <row r="37" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1"/>
     <row r="38" spans="1:8" ht="20.100000000000001" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A38" s="375" t="s">
+      <c r="A38" s="377" t="s">
         <v>953</v>
       </c>
-      <c r="B38" s="376"/>
-      <c r="C38" s="376"/>
-      <c r="D38" s="376"/>
-      <c r="E38" s="376"/>
-      <c r="F38" s="377"/>
+      <c r="B38" s="378"/>
+      <c r="C38" s="378"/>
+      <c r="D38" s="378"/>
+      <c r="E38" s="378"/>
+      <c r="F38" s="379"/>
       <c r="G38" s="175"/>
       <c r="H38" s="175"/>
     </row>
     <row r="39" spans="1:8" ht="20.100000000000001" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A39" s="378" t="s">
+      <c r="A39" s="380" t="s">
         <v>840</v>
       </c>
-      <c r="B39" s="379"/>
-      <c r="C39" s="380"/>
-      <c r="D39" s="378" t="s">
+      <c r="B39" s="381"/>
+      <c r="C39" s="382"/>
+      <c r="D39" s="380" t="s">
         <v>841</v>
       </c>
-      <c r="E39" s="379"/>
-      <c r="F39" s="380"/>
+      <c r="E39" s="381"/>
+      <c r="F39" s="382"/>
       <c r="G39" s="175"/>
       <c r="H39" s="175"/>
     </row>
@@ -19059,7 +19131,7 @@
         <v>1</v>
       </c>
       <c r="G40" s="175"/>
-      <c r="H40" s="369" t="s">
+      <c r="H40" s="371" t="s">
         <v>844</v>
       </c>
     </row>
@@ -19083,7 +19155,7 @@
         <v>2</v>
       </c>
       <c r="G41" s="175"/>
-      <c r="H41" s="370"/>
+      <c r="H41" s="372"/>
     </row>
     <row r="42" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A42" s="204">
@@ -19105,7 +19177,7 @@
         <v>3</v>
       </c>
       <c r="G42" s="175"/>
-      <c r="H42" s="370"/>
+      <c r="H42" s="372"/>
     </row>
     <row r="43" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A43" s="206">
@@ -19127,7 +19199,7 @@
         <v>4</v>
       </c>
       <c r="G43" s="175"/>
-      <c r="H43" s="370"/>
+      <c r="H43" s="372"/>
     </row>
     <row r="44" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A44" s="206">
@@ -19149,7 +19221,7 @@
         <v>5</v>
       </c>
       <c r="G44" s="175"/>
-      <c r="H44" s="370"/>
+      <c r="H44" s="372"/>
     </row>
     <row r="45" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A45" s="208">
@@ -19171,7 +19243,7 @@
         <v>6</v>
       </c>
       <c r="G45" s="175"/>
-      <c r="H45" s="370"/>
+      <c r="H45" s="372"/>
     </row>
     <row r="46" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A46" s="208">
@@ -19193,7 +19265,7 @@
         <v>7</v>
       </c>
       <c r="G46" s="175"/>
-      <c r="H46" s="370"/>
+      <c r="H46" s="372"/>
     </row>
     <row r="47" spans="1:8" ht="20.100000000000001" customHeight="1" thickBot="1">
       <c r="A47" s="210">
@@ -19215,7 +19287,7 @@
         <v>8</v>
       </c>
       <c r="G47" s="175"/>
-      <c r="H47" s="371"/>
+      <c r="H47" s="373"/>
     </row>
     <row r="48" spans="1:8" ht="20.100000000000001" customHeight="1" thickTop="1" thickBot="1">
       <c r="A48" s="213">
@@ -19237,7 +19309,7 @@
         <v>9</v>
       </c>
       <c r="G48" s="175"/>
-      <c r="H48" s="372" t="s">
+      <c r="H48" s="374" t="s">
         <v>856</v>
       </c>
     </row>
@@ -19261,7 +19333,7 @@
         <v>10</v>
       </c>
       <c r="G49" s="175"/>
-      <c r="H49" s="373"/>
+      <c r="H49" s="375"/>
     </row>
     <row r="50" spans="1:8" ht="16.5" thickBot="1">
       <c r="A50" s="215">
@@ -19283,7 +19355,7 @@
         <v>11</v>
       </c>
       <c r="G50" s="175"/>
-      <c r="H50" s="373"/>
+      <c r="H50" s="375"/>
     </row>
     <row r="51" spans="1:8" ht="16.5" thickBot="1">
       <c r="A51" s="218">
@@ -19305,7 +19377,7 @@
         <v>12</v>
       </c>
       <c r="G51" s="175"/>
-      <c r="H51" s="373"/>
+      <c r="H51" s="375"/>
     </row>
     <row r="52" spans="1:8" ht="16.5" thickBot="1">
       <c r="A52" s="218">
@@ -19327,7 +19399,7 @@
         <v>13</v>
       </c>
       <c r="G52" s="175"/>
-      <c r="H52" s="373"/>
+      <c r="H52" s="375"/>
     </row>
     <row r="53" spans="1:8" ht="16.5" thickBot="1">
       <c r="A53" s="218">
@@ -19349,7 +19421,7 @@
         <v>14</v>
       </c>
       <c r="G53" s="175"/>
-      <c r="H53" s="373"/>
+      <c r="H53" s="375"/>
     </row>
     <row r="54" spans="1:8" ht="16.5" thickBot="1">
       <c r="A54" s="218">
@@ -19371,7 +19443,7 @@
         <v>15</v>
       </c>
       <c r="G54" s="175"/>
-      <c r="H54" s="373"/>
+      <c r="H54" s="375"/>
     </row>
     <row r="55" spans="1:8" ht="16.5" thickBot="1">
       <c r="A55" s="218">
@@ -19393,7 +19465,7 @@
         <v>16</v>
       </c>
       <c r="G55" s="175"/>
-      <c r="H55" s="373"/>
+      <c r="H55" s="375"/>
     </row>
     <row r="56" spans="1:8" ht="16.5" thickBot="1">
       <c r="A56" s="218">
@@ -19415,7 +19487,7 @@
         <v>17</v>
       </c>
       <c r="G56" s="175"/>
-      <c r="H56" s="373"/>
+      <c r="H56" s="375"/>
     </row>
     <row r="57" spans="1:8" ht="16.5" thickBot="1">
       <c r="A57" s="220">
@@ -19437,7 +19509,7 @@
         <v>18</v>
       </c>
       <c r="G57" s="175"/>
-      <c r="H57" s="373"/>
+      <c r="H57" s="375"/>
     </row>
     <row r="58" spans="1:8" ht="16.5" thickBot="1">
       <c r="A58" s="220">
@@ -19459,7 +19531,7 @@
         <v>19</v>
       </c>
       <c r="G58" s="175"/>
-      <c r="H58" s="373"/>
+      <c r="H58" s="375"/>
     </row>
     <row r="59" spans="1:8" ht="16.5" thickBot="1">
       <c r="A59" s="222">
@@ -19481,7 +19553,7 @@
         <v>20</v>
       </c>
       <c r="G59" s="175"/>
-      <c r="H59" s="374"/>
+      <c r="H59" s="376"/>
     </row>
     <row r="60" spans="1:8" ht="15.75" thickTop="1"/>
   </sheetData>
@@ -19519,40 +19591,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1">
-      <c r="A1" s="387" t="s">
+      <c r="A1" s="389" t="s">
         <v>327</v>
       </c>
-      <c r="B1" s="388"/>
-      <c r="C1" s="388"/>
-      <c r="D1" s="388"/>
-      <c r="E1" s="388"/>
-      <c r="F1" s="388"/>
-      <c r="G1" s="388"/>
-      <c r="H1" s="389"/>
+      <c r="B1" s="390"/>
+      <c r="C1" s="390"/>
+      <c r="D1" s="390"/>
+      <c r="E1" s="390"/>
+      <c r="F1" s="390"/>
+      <c r="G1" s="390"/>
+      <c r="H1" s="391"/>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1" thickBot="1">
-      <c r="A2" s="390"/>
-      <c r="B2" s="391"/>
-      <c r="C2" s="391"/>
-      <c r="D2" s="391"/>
-      <c r="E2" s="391"/>
-      <c r="F2" s="391"/>
-      <c r="G2" s="391"/>
-      <c r="H2" s="392"/>
+      <c r="A2" s="392"/>
+      <c r="B2" s="393"/>
+      <c r="C2" s="393"/>
+      <c r="D2" s="393"/>
+      <c r="E2" s="393"/>
+      <c r="F2" s="393"/>
+      <c r="G2" s="393"/>
+      <c r="H2" s="394"/>
     </row>
     <row r="3" spans="1:8" ht="21" thickBot="1">
-      <c r="A3" s="381" t="s">
+      <c r="A3" s="383" t="s">
         <v>221</v>
       </c>
-      <c r="B3" s="382"/>
-      <c r="C3" s="382"/>
-      <c r="D3" s="383"/>
-      <c r="E3" s="381" t="s">
+      <c r="B3" s="384"/>
+      <c r="C3" s="384"/>
+      <c r="D3" s="385"/>
+      <c r="E3" s="383" t="s">
         <v>314</v>
       </c>
-      <c r="F3" s="382"/>
-      <c r="G3" s="382"/>
-      <c r="H3" s="383"/>
+      <c r="F3" s="384"/>
+      <c r="G3" s="384"/>
+      <c r="H3" s="385"/>
     </row>
     <row r="4" spans="1:8" ht="17.25" thickBot="1">
       <c r="A4" s="77">
@@ -19769,18 +19841,18 @@
       <c r="H21" s="69"/>
     </row>
     <row r="22" spans="1:8" ht="20.25" thickBot="1">
-      <c r="A22" s="384" t="s">
+      <c r="A22" s="386" t="s">
         <v>315</v>
       </c>
-      <c r="B22" s="385"/>
-      <c r="C22" s="385"/>
-      <c r="D22" s="386"/>
-      <c r="E22" s="384" t="s">
+      <c r="B22" s="387"/>
+      <c r="C22" s="387"/>
+      <c r="D22" s="388"/>
+      <c r="E22" s="386" t="s">
         <v>316</v>
       </c>
-      <c r="F22" s="385"/>
-      <c r="G22" s="385"/>
-      <c r="H22" s="386"/>
+      <c r="F22" s="387"/>
+      <c r="G22" s="387"/>
+      <c r="H22" s="388"/>
     </row>
     <row r="23" spans="1:8" ht="16.5" thickBot="1">
       <c r="A23" s="62">
@@ -20052,40 +20124,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" s="325" t="s">
+      <c r="A1" s="327" t="s">
         <v>488</v>
       </c>
-      <c r="B1" s="326"/>
-      <c r="C1" s="326"/>
-      <c r="D1" s="326"/>
-      <c r="E1" s="326"/>
-      <c r="F1" s="326"/>
-      <c r="G1" s="326"/>
-      <c r="H1" s="327"/>
+      <c r="B1" s="328"/>
+      <c r="C1" s="328"/>
+      <c r="D1" s="328"/>
+      <c r="E1" s="328"/>
+      <c r="F1" s="328"/>
+      <c r="G1" s="328"/>
+      <c r="H1" s="329"/>
     </row>
     <row r="2" spans="1:8" ht="15.75" customHeight="1">
-      <c r="A2" s="328"/>
-      <c r="B2" s="329"/>
-      <c r="C2" s="329"/>
-      <c r="D2" s="329"/>
-      <c r="E2" s="329"/>
-      <c r="F2" s="329"/>
-      <c r="G2" s="329"/>
-      <c r="H2" s="330"/>
+      <c r="A2" s="330"/>
+      <c r="B2" s="331"/>
+      <c r="C2" s="331"/>
+      <c r="D2" s="331"/>
+      <c r="E2" s="331"/>
+      <c r="F2" s="331"/>
+      <c r="G2" s="331"/>
+      <c r="H2" s="332"/>
     </row>
     <row r="3" spans="1:8" ht="19.5" customHeight="1">
-      <c r="A3" s="331" t="s">
+      <c r="A3" s="333" t="s">
         <v>319</v>
       </c>
-      <c r="B3" s="332"/>
-      <c r="C3" s="332"/>
-      <c r="D3" s="332"/>
-      <c r="E3" s="332" t="s">
+      <c r="B3" s="334"/>
+      <c r="C3" s="334"/>
+      <c r="D3" s="334"/>
+      <c r="E3" s="334" t="s">
         <v>318</v>
       </c>
-      <c r="F3" s="332"/>
-      <c r="G3" s="332"/>
-      <c r="H3" s="333"/>
+      <c r="F3" s="334"/>
+      <c r="G3" s="334"/>
+      <c r="H3" s="335"/>
     </row>
     <row r="4" spans="1:8" ht="18.75" thickBot="1">
       <c r="A4" s="12">

</xml_diff>